<commit_message>
Regenerate AllYears combined file with cleaned 2013/2014 data
Re-ran combine_all_years.py after the 2013/2014 pipeline rebuild.

Top-level changes vs the previous combined snapshot:
- 2013 row count: 15 → 17  (PIPL 116 → 95, banded 53 → 2)
- 2014 row count: 65 → 100 (PIPL 398 → 371, banded 0 → 46)
- Total rows:    1093 → 1130
- Total PIPL:    3550 → 3502  (more accurate — 2013 was over-counting)
- Banded:        496  → 491   (2013 corrected; 2014 newly populated)

The 2014 FlagCode column is now empty across all 100 rows (previously
contained band data that should have been in BandCombo). 2014 BandCombo
column is now populated with 46 banded entries reflecting the biologist
review corrections.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Databases/Database3/Output/AllYears/db3_2013_FINAL.xlsx
+++ b/Databases/Database3/Output/AllYears/db3_2013_FINAL.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Clean_Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Removed_Rows" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary_Report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean_Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed_Rows" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_Report" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,23 +458,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="46" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="31" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="46" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="31" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,60 +494,80 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>SurveyTime</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>WeatherCondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>GroupNumber</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>TotalObserved</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Observer</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ObserverEmail</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>FlagCode</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>FlagColor</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>BandCombo</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>source_database</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>source_sheet</t>
         </is>
@@ -556,52 +580,52 @@
       <c r="B2" s="2" t="n">
         <v>41313</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Anclote Key- north route</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>28.214</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>-82.84699999999999</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="n">
         <v>8</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>DLarremore, CMaxwell, ACornett</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>daniel.larremore@dep.state.fl.us</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
         <is>
           <t>1 banded PIPL seen, flushed before reading</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -614,44 +638,48 @@
       <c r="B3" s="2" t="n">
         <v>41313</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Anclote Key- south route</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>28.1593</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>-82.8434</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="n">
         <v>46</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>LKenney, TCarey, SArmstrong</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>likenney@aol.com</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -664,48 +692,48 @@
       <c r="B4" s="2" t="n">
         <v>41306</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Big Marco Pass CWA</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>25.95291</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>-81.75093</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="n">
         <v>5</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>RZambrano, CRizkalla</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>ricardo.zambrano@myfwc.om</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -718,48 +746,48 @@
       <c r="B5" s="2" t="n">
         <v>41315</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Honeymoon Island- north route</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="F5" t="n">
         <v>28.0926</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>-82.8361</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="n">
         <v>2</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>DLarremore, LKinney</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>daniel.larremore@dep.state.fl.us</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -772,48 +800,48 @@
       <c r="B6" s="2" t="n">
         <v>41315</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Honeymoon Island- north route</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="F6" t="n">
         <v>28.0937</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>-82.83620000000001</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="n">
         <v>2</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>DLarremore, LKinney</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>daniel.larremore@dep.state.fl.us</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -826,50 +854,52 @@
       <c r="B7" s="2" t="n">
         <v>41315</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Honeymoon Island- north route</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="F7" t="n">
         <v>28.0947</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>-82.8361</v>
       </c>
-      <c r="F7" t="n">
-        <v>8</v>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>DLarremore, LKinney</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>daniel.larremore@dep.state.fl.us</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
         <is>
           <t>left- Green flag above, 0 below. right-green band above, white over orange below</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -882,48 +912,48 @@
       <c r="B8" s="2" t="n">
         <v>41315</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Honeymoon Island- north route</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>28.0979</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-82.83540000000001</v>
-      </c>
       <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
+        <v>28.0947</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-82.8361</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>DLarremore, LKinney</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>daniel.larremore@dep.state.fl.us</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -936,48 +966,48 @@
       <c r="B9" s="2" t="n">
         <v>41315</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Honeymoon Island- north route</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>28.0984</v>
-      </c>
-      <c r="E9" t="n">
-        <v>-82.8349</v>
-      </c>
       <c r="F9" t="n">
+        <v>28.0979</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-82.83540000000001</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>DLarremore, LKinney</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>daniel.larremore@dep.state.fl.us</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -988,46 +1018,50 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>41311</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Mid-Fort De Soto Rte 1</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>27.62014</v>
-      </c>
-      <c r="E10" t="n">
-        <v>-82.73668000000001</v>
+        <v>41315</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Honeymoon Island- north route</t>
+        </is>
       </c>
       <c r="F10" t="n">
+        <v>28.0984</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-82.8349</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Nancy Ogden</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>verdnan23@gmail.com</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>DLarremore, LKinney</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>daniel.larremore@dep.state.fl.us</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -1038,54 +1072,50 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>41313</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>North Anclote Bar</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>28.2337</v>
-      </c>
-      <c r="E11" t="n">
-        <v>-82.839</v>
+        <v>41311</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mid-Fort De Soto Rte 1</t>
+        </is>
       </c>
       <c r="F11" t="n">
-        <v>16</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>DGagne, BPranty</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>oporornis77@yahoo.com</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>REKN- 2 w/  green flags, no codes reported. PIPL- green flag</t>
-        </is>
+        <v>27.62014</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-82.73668000000001</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>1</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>left- 0 above, orange over blue below. right- green flag above, yellow over silver below.</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
+          <t>Nancy Ogden</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>verdnan23@gmail.com</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -1098,52 +1128,52 @@
       <c r="B12" s="2" t="n">
         <v>41313</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>North Rockhouse Creek Shoals island, Ponce Inlet</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>29.069715947</v>
-      </c>
-      <c r="E12" t="n">
-        <v>-80.92578097000001</v>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>North Anclote Bar</t>
+        </is>
       </c>
       <c r="F12" t="n">
-        <v>8</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>J.Winters, J. Milio, M. Wilson</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>jwinters@volusia.org</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>n/A</t>
-        </is>
+        <v>28.2337</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-82.839</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>1</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>none banded</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
+          <t>DGagne, BPranty</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>oporornis77@yahoo.com</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>green flag | left- 0 above, orange over blue below. right- green flag above, yellow over silver below</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -1156,48 +1186,48 @@
       <c r="B13" s="2" t="n">
         <v>41313</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>North Rockhouse Creek Shoals island, Ponce Inlet</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>29.06983032</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-80.92578097000001</v>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>North Anclote Bar</t>
+        </is>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>J. Winters, J. Milio, M. Wilson</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>jwinters@volusia.org</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+        <v>28.2337</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-82.839</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>15</v>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>none banded</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
+          <t>DGagne, BPranty</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>oporornis77@yahoo.com</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -1210,44 +1240,48 @@
       <c r="B14" s="2" t="n">
         <v>41313</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">South Volusia County; Indian River Lagoon </t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>28.570137</v>
-      </c>
-      <c r="E14" t="n">
-        <v>-80.874516</v>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>North Rockhouse Creek Shoals island, Ponce Inlet</t>
+        </is>
       </c>
       <c r="F14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Ken Gunn, Don Picard</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>gunnsatbeach@cfl.rr.com</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
+        <v>29.069715947</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-80.92578097000001</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>J.Winters, J. Milio, M. Wilson</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>jwinters@volusia.org</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -1260,44 +1294,48 @@
       <c r="B15" s="2" t="n">
         <v>41313</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">South Volusia County; Indian River Lagoon </t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>29.001266</v>
-      </c>
-      <c r="E15" t="n">
-        <v>-80.90001599999999</v>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>North Rockhouse Creek Shoals island, Ponce Inlet</t>
+        </is>
       </c>
       <c r="F15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Ken Gunn, Don Picard</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>gunnsatbeach@cfl.rr.com</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
+        <v>29.06983032</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-80.92578097000001</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>J. Winters, J. Milio, M. Wilson</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>jwinters@volusia.org</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -1308,50 +1346,162 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="n">
+        <v>41313</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>South Volusia County; Indian River Lagoon</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>28.570137</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-80.874516</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Ken Gunn, Don Picard</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>gunnsatbeach@cfl.rr.com</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>WinterBirdSurvey</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Winter Birds '13 Clean.xlsx</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Species GPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>41313</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>South Volusia County; Indian River Lagoon</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>29.001266</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-80.90001599999999</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Ken Gunn, Don Picard</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>gunnsatbeach@cfl.rr.com</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>WinterBirdSurvey</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Winter Birds '13 Clean.xlsx</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Species GPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="n">
         <v>41381</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Mid-Fort De Soto Rte 1</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="F18" t="n">
         <v>27.61177</v>
       </c>
-      <c r="E16" t="n">
+      <c r="G18" t="n">
         <v>-82.73617</v>
       </c>
-      <c r="F16" t="n">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
         <v>1</v>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Nancy Ogden</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>verdnan23@gmail.com</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
         <is>
           <t>High up on beach close to dunes</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>Winter Birds '13 Clean.xlsx</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>Species GPS</t>
         </is>
@@ -1425,7 +1575,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-18 12:14</t>
+          <t>2026-06-26 10:18</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1630,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1522,7 +1672,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
@@ -1650,7 +1800,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  unique_id 9</t>
+          <t xml:space="preserve">  unique_id 10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1662,7 +1812,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  unique_id 15</t>
+          <t xml:space="preserve">  unique_id 17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">

</xml_diff>